<commit_message>
codul de baza pt metoda jacobi si gauss-seidel
</commit_message>
<xml_diff>
--- a/Calcul Numeric/Prezenta.xlsx
+++ b/Calcul Numeric/Prezenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Facultate_Promotia_2024_2027\Calcul Numeric\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B248CF2-3991-4D63-85E1-D03D143F7B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FD6F9D-D3D7-4818-B965-A4FCD49269AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -262,6 +262,12 @@
   </si>
   <si>
     <t>Razvan Magui</t>
+  </si>
+  <si>
+    <t>Rafael Foica</t>
+  </si>
+  <si>
+    <t>Teodora Borze</t>
   </si>
 </sst>
 </file>
@@ -481,7 +487,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -531,22 +537,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Default" xfId="1" xr:uid="{C2A1F133-5CCB-48A4-A954-37FCB6A8888E}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -835,7 +831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:R64"/>
+  <dimension ref="B2:R66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="2" customWidth="1"/>
@@ -915,7 +911,7 @@
       <c r="O3" s="5"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="4">
-        <f>COUNT(C3:P3)</f>
+        <f t="shared" ref="Q3:Q34" si="0">COUNT(C3:P3)</f>
         <v>0</v>
       </c>
       <c r="R3" s="12" t="str">
@@ -930,25 +926,16 @@
       <c r="C4" s="7">
         <v>2</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
       <c r="P4" s="8"/>
       <c r="Q4" s="7">
-        <f>COUNT(C4:P4)</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="R4" s="13">
-        <f t="shared" ref="R4:R64" si="0">IF(COUNT(C4:P4)&gt;0, MIN(5+(COUNTIF(C4:P4,"&gt;1")/2),10), "absent")</f>
+        <f t="shared" ref="R4:R64" si="1">IF(COUNT(C4:P4)&gt;0, MIN(5+(COUNTIF(C4:P4,"&gt;1")/2),10), "absent")</f>
         <v>5.5</v>
       </c>
     </row>
@@ -959,25 +946,13 @@
       <c r="C5" s="7">
         <v>2</v>
       </c>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
       <c r="P5" s="8"/>
       <c r="Q5" s="7">
-        <f>COUNT(C5:P5)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -988,25 +963,13 @@
       <c r="C6" s="7">
         <v>2</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="7">
-        <f>COUNT(C6:P6)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R6" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1017,25 +980,16 @@
       <c r="C7" s="7">
         <v>2</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
       <c r="P7" s="8"/>
       <c r="Q7" s="7">
-        <f>COUNT(C7:P7)</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="R7" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1046,25 +1000,13 @@
       <c r="C8" s="7">
         <v>2</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="7">
-        <f>COUNT(C8:P8)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R8" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1075,25 +1017,13 @@
       <c r="C9" s="7">
         <v>2</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
       <c r="P9" s="8"/>
       <c r="Q9" s="7">
-        <f>COUNT(C9:P9)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R9" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1102,25 +1032,13 @@
         <v>47</v>
       </c>
       <c r="C10" s="7"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="17"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="7">
-        <f>COUNT(C10:P10)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R10" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1129,25 +1047,13 @@
         <v>67</v>
       </c>
       <c r="C11" s="7"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="7">
-        <f>COUNT(C11:P11)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R11" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1156,25 +1062,13 @@
         <v>32</v>
       </c>
       <c r="C12" s="7"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
       <c r="P12" s="8"/>
       <c r="Q12" s="7">
-        <f>COUNT(C12:P12)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R12" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1185,25 +1079,16 @@
       <c r="C13" s="7">
         <v>2</v>
       </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
-      <c r="O13" s="17"/>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
       <c r="P13" s="8"/>
       <c r="Q13" s="7">
-        <f>COUNT(C13:P13)</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="R13" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1212,26 +1097,17 @@
         <v>70</v>
       </c>
       <c r="C14" s="7"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
       <c r="P14" s="8"/>
       <c r="Q14" s="7">
-        <f>COUNT(C14:P14)</f>
-        <v>0</v>
-      </c>
-      <c r="R14" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>absent</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="R14" s="13">
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="2:18">
@@ -1239,25 +1115,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="7"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
-      <c r="O15" s="17"/>
       <c r="P15" s="8"/>
       <c r="Q15" s="7">
-        <f>COUNT(C15:P15)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R15" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1268,25 +1132,13 @@
       <c r="C16" s="7">
         <v>2</v>
       </c>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
       <c r="P16" s="8"/>
       <c r="Q16" s="7">
-        <f>COUNT(C16:P16)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R16" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1297,25 +1149,16 @@
       <c r="C17" s="7">
         <v>2</v>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
       <c r="P17" s="8"/>
       <c r="Q17" s="7">
-        <f>COUNT(C17:P17)</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="R17" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1324,25 +1167,13 @@
         <v>55</v>
       </c>
       <c r="C18" s="7"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
       <c r="P18" s="8"/>
       <c r="Q18" s="7">
-        <f>COUNT(C18:P18)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R18" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1351,25 +1182,13 @@
         <v>33</v>
       </c>
       <c r="C19" s="7"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
       <c r="P19" s="8"/>
       <c r="Q19" s="7">
-        <f>COUNT(C19:P19)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R19" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1378,25 +1197,13 @@
         <v>69</v>
       </c>
       <c r="C20" s="7"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
       <c r="P20" s="8"/>
       <c r="Q20" s="7">
-        <f>COUNT(C20:P20)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R20" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1405,25 +1212,13 @@
         <v>26</v>
       </c>
       <c r="C21" s="7"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
       <c r="P21" s="8"/>
       <c r="Q21" s="7">
-        <f>COUNT(C21:P21)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R21" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1432,25 +1227,13 @@
         <v>22</v>
       </c>
       <c r="C22" s="7"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
       <c r="P22" s="8"/>
       <c r="Q22" s="7">
-        <f>COUNT(C22:P22)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R22" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1459,25 +1242,13 @@
         <v>50</v>
       </c>
       <c r="C23" s="7"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
       <c r="P23" s="8"/>
       <c r="Q23" s="7">
-        <f>COUNT(C23:P23)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R23" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1488,25 +1259,13 @@
       <c r="C24" s="7">
         <v>2</v>
       </c>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
-      <c r="M24" s="17"/>
-      <c r="N24" s="17"/>
-      <c r="O24" s="17"/>
       <c r="P24" s="8"/>
       <c r="Q24" s="7">
-        <f>COUNT(C24:P24)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R24" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1515,25 +1274,13 @@
         <v>49</v>
       </c>
       <c r="C25" s="7"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
-      <c r="O25" s="17"/>
       <c r="P25" s="8"/>
       <c r="Q25" s="7">
-        <f>COUNT(C25:P25)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R25" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1542,25 +1289,13 @@
         <v>64</v>
       </c>
       <c r="C26" s="7"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
-      <c r="O26" s="17"/>
       <c r="P26" s="8"/>
       <c r="Q26" s="7">
-        <f>COUNT(C26:P26)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R26" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1569,25 +1304,13 @@
         <v>36</v>
       </c>
       <c r="C27" s="7"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="17"/>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
-      <c r="O27" s="17"/>
       <c r="P27" s="8"/>
       <c r="Q27" s="7">
-        <f>COUNT(C27:P27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R27" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1598,25 +1321,13 @@
       <c r="C28" s="7">
         <v>2</v>
       </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
       <c r="P28" s="8"/>
       <c r="Q28" s="7">
-        <f>COUNT(C28:P28)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R28" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1627,25 +1338,13 @@
       <c r="C29" s="7">
         <v>2</v>
       </c>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="17"/>
       <c r="P29" s="8"/>
       <c r="Q29" s="7">
-        <f>COUNT(C29:P29)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R29" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1656,25 +1355,16 @@
       <c r="C30" s="7">
         <v>2</v>
       </c>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
-      <c r="M30" s="17"/>
-      <c r="N30" s="17"/>
-      <c r="O30" s="17"/>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
       <c r="P30" s="8"/>
       <c r="Q30" s="7">
-        <f>COUNT(C30:P30)</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="R30" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1683,25 +1373,13 @@
         <v>61</v>
       </c>
       <c r="C31" s="7"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
       <c r="P31" s="8"/>
       <c r="Q31" s="7">
-        <f>COUNT(C31:P31)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R31" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1710,25 +1388,13 @@
         <v>43</v>
       </c>
       <c r="C32" s="7"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="17"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="17"/>
       <c r="P32" s="8"/>
       <c r="Q32" s="7">
-        <f>COUNT(C32:P32)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R32" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1739,25 +1405,13 @@
       <c r="C33" s="7">
         <v>2</v>
       </c>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
-      <c r="O33" s="17"/>
       <c r="P33" s="8"/>
       <c r="Q33" s="7">
-        <f>COUNT(C33:P33)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R33" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1768,25 +1422,13 @@
       <c r="C34" s="7">
         <v>2</v>
       </c>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
-      <c r="O34" s="17"/>
       <c r="P34" s="8"/>
       <c r="Q34" s="7">
-        <f>COUNT(C34:P34)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="R34" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1795,25 +1437,13 @@
         <v>58</v>
       </c>
       <c r="C35" s="7"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
-      <c r="M35" s="17"/>
-      <c r="N35" s="17"/>
-      <c r="O35" s="17"/>
       <c r="P35" s="8"/>
       <c r="Q35" s="7">
-        <f>COUNT(C35:P35)</f>
+        <f t="shared" ref="Q35:Q66" si="2">COUNT(C35:P35)</f>
         <v>0</v>
       </c>
       <c r="R35" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1822,25 +1452,13 @@
         <v>62</v>
       </c>
       <c r="C36" s="7"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
       <c r="P36" s="8"/>
       <c r="Q36" s="7">
-        <f>COUNT(C36:P36)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R36" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1851,25 +1469,13 @@
       <c r="C37" s="7">
         <v>2</v>
       </c>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
       <c r="P37" s="8"/>
       <c r="Q37" s="7">
-        <f>COUNT(C37:P37)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R37" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -1878,25 +1484,13 @@
         <v>54</v>
       </c>
       <c r="C38" s="7"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-      <c r="N38" s="17"/>
-      <c r="O38" s="17"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="7">
-        <f>COUNT(C38:P38)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R38" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1905,25 +1499,13 @@
         <v>57</v>
       </c>
       <c r="C39" s="7"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="7">
-        <f>COUNT(C39:P39)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R39" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1932,25 +1514,13 @@
         <v>27</v>
       </c>
       <c r="C40" s="7"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
       <c r="P40" s="8"/>
       <c r="Q40" s="7">
-        <f>COUNT(C40:P40)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R40" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1959,25 +1529,13 @@
         <v>19</v>
       </c>
       <c r="C41" s="7"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
       <c r="P41" s="8"/>
       <c r="Q41" s="7">
-        <f>COUNT(C41:P41)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R41" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -1988,25 +1546,16 @@
       <c r="C42" s="7">
         <v>2</v>
       </c>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
-      <c r="K42" s="17"/>
-      <c r="L42" s="17"/>
-      <c r="M42" s="17"/>
-      <c r="N42" s="17"/>
-      <c r="O42" s="17"/>
+      <c r="D42" s="2">
+        <v>1</v>
+      </c>
       <c r="P42" s="8"/>
       <c r="Q42" s="7">
-        <f>COUNT(C42:P42)</f>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="R42" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2017,25 +1566,13 @@
       <c r="C43" s="7">
         <v>2</v>
       </c>
-      <c r="D43" s="17"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
       <c r="P43" s="8"/>
       <c r="Q43" s="7">
-        <f>COUNT(C43:P43)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R43" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2046,25 +1583,13 @@
       <c r="C44" s="7">
         <v>2</v>
       </c>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
-      <c r="O44" s="17"/>
       <c r="P44" s="8"/>
       <c r="Q44" s="7">
-        <f>COUNT(C44:P44)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R44" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2075,25 +1600,13 @@
       <c r="C45" s="7">
         <v>2</v>
       </c>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
       <c r="P45" s="8"/>
       <c r="Q45" s="7">
-        <f>COUNT(C45:P45)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R45" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2102,25 +1615,13 @@
         <v>44</v>
       </c>
       <c r="C46" s="7"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
       <c r="P46" s="8"/>
       <c r="Q46" s="7">
-        <f>COUNT(C46:P46)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R46" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2131,25 +1632,13 @@
       <c r="C47" s="7">
         <v>2</v>
       </c>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
       <c r="P47" s="8"/>
       <c r="Q47" s="7">
-        <f>COUNT(C47:P47)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R47" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2160,25 +1649,16 @@
       <c r="C48" s="7">
         <v>2</v>
       </c>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
+      <c r="D48" s="2">
+        <v>1</v>
+      </c>
       <c r="P48" s="8"/>
       <c r="Q48" s="7">
-        <f>COUNT(C48:P48)</f>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="R48" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2189,25 +1669,13 @@
       <c r="C49" s="7">
         <v>2</v>
       </c>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
       <c r="P49" s="8"/>
       <c r="Q49" s="7">
-        <f>COUNT(C49:P49)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R49" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2218,25 +1686,13 @@
       <c r="C50" s="7">
         <v>2</v>
       </c>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
       <c r="P50" s="8"/>
       <c r="Q50" s="7">
-        <f>COUNT(C50:P50)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R50" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2247,25 +1703,13 @@
       <c r="C51" s="7">
         <v>2</v>
       </c>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17"/>
-      <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
       <c r="P51" s="8"/>
       <c r="Q51" s="7">
-        <f>COUNT(C51:P51)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R51" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2274,25 +1718,13 @@
         <v>39</v>
       </c>
       <c r="C52" s="7"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
       <c r="P52" s="8"/>
       <c r="Q52" s="7">
-        <f>COUNT(C52:P52)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R52" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2303,25 +1735,13 @@
       <c r="C53" s="7">
         <v>2</v>
       </c>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
       <c r="P53" s="8"/>
       <c r="Q53" s="7">
-        <f>COUNT(C53:P53)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R53" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2332,25 +1752,13 @@
       <c r="C54" s="7">
         <v>2</v>
       </c>
-      <c r="D54" s="17"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
       <c r="P54" s="8"/>
       <c r="Q54" s="7">
-        <f>COUNT(C54:P54)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R54" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2361,25 +1769,13 @@
       <c r="C55" s="7">
         <v>2</v>
       </c>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
       <c r="P55" s="8"/>
       <c r="Q55" s="7">
-        <f>COUNT(C55:P55)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R55" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2388,26 +1784,17 @@
         <v>66</v>
       </c>
       <c r="C56" s="7"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="17"/>
-      <c r="G56" s="17"/>
-      <c r="H56" s="17"/>
-      <c r="I56" s="17"/>
-      <c r="J56" s="17"/>
-      <c r="K56" s="17"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
+      <c r="D56" s="2">
+        <v>1</v>
+      </c>
       <c r="P56" s="8"/>
       <c r="Q56" s="7">
-        <f>COUNT(C56:P56)</f>
-        <v>0</v>
-      </c>
-      <c r="R56" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>absent</v>
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="R56" s="13">
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
     </row>
     <row r="57" spans="2:18">
@@ -2417,25 +1804,16 @@
       <c r="C57" s="7">
         <v>2</v>
       </c>
-      <c r="D57" s="17"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
+      <c r="D57" s="2">
+        <v>1</v>
+      </c>
       <c r="P57" s="8"/>
       <c r="Q57" s="7">
-        <f>COUNT(C57:P57)</f>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="R57" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2444,25 +1822,13 @@
         <v>48</v>
       </c>
       <c r="C58" s="7"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="17"/>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
       <c r="P58" s="8"/>
       <c r="Q58" s="7">
-        <f>COUNT(C58:P58)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R58" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2471,25 +1837,13 @@
         <v>52</v>
       </c>
       <c r="C59" s="7"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
-      <c r="N59" s="17"/>
-      <c r="O59" s="17"/>
       <c r="P59" s="8"/>
       <c r="Q59" s="7">
-        <f>COUNT(C59:P59)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R59" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2500,25 +1854,16 @@
       <c r="C60" s="7">
         <v>2</v>
       </c>
-      <c r="D60" s="17"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="17"/>
-      <c r="I60" s="17"/>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
-      <c r="L60" s="17"/>
-      <c r="M60" s="17"/>
-      <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
+      <c r="D60" s="2">
+        <v>1</v>
+      </c>
       <c r="P60" s="8"/>
       <c r="Q60" s="7">
-        <f>COUNT(C60:P60)</f>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="R60" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
@@ -2527,26 +1872,17 @@
         <v>46</v>
       </c>
       <c r="C61" s="7"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-      <c r="G61" s="17"/>
-      <c r="H61" s="17"/>
-      <c r="I61" s="17"/>
-      <c r="J61" s="17"/>
-      <c r="K61" s="17"/>
-      <c r="L61" s="17"/>
-      <c r="M61" s="17"/>
-      <c r="N61" s="17"/>
-      <c r="O61" s="17"/>
+      <c r="D61" s="2">
+        <v>1</v>
+      </c>
       <c r="P61" s="8"/>
       <c r="Q61" s="7">
-        <f>COUNT(C61:P61)</f>
-        <v>0</v>
-      </c>
-      <c r="R61" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>absent</v>
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="R61" s="13">
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="2:18">
@@ -2554,25 +1890,13 @@
         <v>45</v>
       </c>
       <c r="C62" s="7"/>
-      <c r="D62" s="17"/>
-      <c r="E62" s="17"/>
-      <c r="F62" s="17"/>
-      <c r="G62" s="17"/>
-      <c r="H62" s="17"/>
-      <c r="I62" s="17"/>
-      <c r="J62" s="17"/>
-      <c r="K62" s="17"/>
-      <c r="L62" s="17"/>
-      <c r="M62" s="17"/>
-      <c r="N62" s="17"/>
-      <c r="O62" s="17"/>
       <c r="P62" s="8"/>
       <c r="Q62" s="7">
-        <f>COUNT(C62:P62)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R62" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2581,25 +1905,13 @@
         <v>29</v>
       </c>
       <c r="C63" s="7"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-      <c r="G63" s="17"/>
-      <c r="H63" s="17"/>
-      <c r="I63" s="17"/>
-      <c r="J63" s="17"/>
-      <c r="K63" s="17"/>
-      <c r="L63" s="17"/>
-      <c r="M63" s="17"/>
-      <c r="N63" s="17"/>
-      <c r="O63" s="17"/>
       <c r="P63" s="8"/>
       <c r="Q63" s="7">
-        <f>COUNT(C63:P63)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R63" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>absent</v>
       </c>
     </row>
@@ -2622,24 +1934,51 @@
       <c r="O64" s="10"/>
       <c r="P64" s="11"/>
       <c r="Q64" s="9">
-        <f>COUNT(C64:P64)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R64" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>absent</v>
+        <f t="shared" si="1"/>
+        <v>absent</v>
+      </c>
+    </row>
+    <row r="65" spans="2:18">
+      <c r="B65" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D65" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q65" s="9">
+        <f t="shared" ref="Q65:Q66" si="3">COUNT(C65:P65)</f>
+        <v>1</v>
+      </c>
+      <c r="R65" s="14">
+        <f t="shared" ref="R65:R66" si="4">IF(COUNT(C65:P65)&gt;0, MIN(5+(COUNTIF(C65:P65,"&gt;1")/2),10), "absent")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="2:18">
+      <c r="B66" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D66" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q66" s="9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="R66" s="14">
+        <f t="shared" si="4"/>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R64">
     <sortCondition ref="B64"/>
   </sortState>
-  <conditionalFormatting sqref="C3:P63">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThanOrEqual">
-      <formula>2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C64:P64">
+  <conditionalFormatting sqref="C3:P64">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>

</xml_diff>